<commit_message>
Updated Standings, Box Scores, Old Template Issue
Data Input for Standings and Box Scores to EOD 9/30/26, fixed old Arizona team being included in Standings template
</commit_message>
<xml_diff>
--- a/2026-2027/BoxScores/April.xlsx
+++ b/2026-2027/BoxScores/April.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\NHLStats\2026-2027\BoxScores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D10BB54-585E-4E3C-B259-EE011CBF8648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82FEDA93-C2E2-42CA-B93C-3AC57003F52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="1590" windowWidth="38640" windowHeight="15720" xr2:uid="{7901B5C0-98B5-4042-9E0B-86E022D78A84}"/>
   </bookViews>
@@ -158,9 +158,6 @@
     <t>Boston Bruins</t>
   </si>
   <si>
-    <t>Arizona Coyotes</t>
-  </si>
-  <si>
     <t>Anaheim Ducks</t>
   </si>
   <si>
@@ -339,6 +336,9 @@
   </si>
   <si>
     <t>April 10th, 2026</t>
+  </si>
+  <si>
+    <t>Utah Mammoth</t>
   </si>
 </sst>
 </file>
@@ -975,206 +975,206 @@
   <sheetData>
     <row r="1" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B1" s="20"/>
       <c r="AA1" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A2" s="14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" s="15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" s="15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA7" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="AA8" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" s="15" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" s="15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="11" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="AA12" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="AA13" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="AA14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="AA15" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="AA16" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA17" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA18" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA19" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA20" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA21" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA22" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA23" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA24" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="25" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA25" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA26" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA27" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="27:27" x14ac:dyDescent="0.3">
       <c r="AA28" s="1" t="s">
-        <v>4</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="27:27" x14ac:dyDescent="0.3">
@@ -1233,33 +1233,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -1354,12 +1354,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1406,33 +1406,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -1527,12 +1527,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -1580,67 +1580,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1665,43 +1665,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -1746,67 +1746,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1831,43 +1831,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -1912,67 +1912,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1997,43 +1997,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2078,67 +2078,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2163,43 +2163,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2243,33 +2243,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -2364,12 +2364,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -2417,67 +2417,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2502,43 +2502,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2583,67 +2583,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2668,43 +2668,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2749,67 +2749,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2834,43 +2834,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2915,67 +2915,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -3000,43 +3000,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -3081,67 +3081,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -3166,43 +3166,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -3246,33 +3246,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -3367,12 +3367,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -3420,67 +3420,67 @@
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="P1" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="U1" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P1" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q1" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="U1" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -3505,43 +3505,43 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -3585,33 +3585,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -3706,12 +3706,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -3758,33 +3758,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -3879,12 +3879,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -3931,33 +3931,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -4052,12 +4052,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -4104,33 +4104,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -4225,12 +4225,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -4277,33 +4277,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -4398,12 +4398,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -4450,33 +4450,33 @@
   <sheetData>
     <row r="1" spans="1:27" ht="22.2" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B1" s="21"/>
       <c r="C1" s="21"/>
       <c r="D1" s="21"/>
       <c r="E1" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:27" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>36</v>
-      </c>
       <c r="D2" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AA2" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -4571,12 +4571,12 @@
     </row>
     <row r="18" spans="1:4" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>